<commit_message>
feat: enhance Excel file handling with styled headers and summary calculations
</commit_message>
<xml_diff>
--- a/components/steam_data.xlsx
+++ b/components/steam_data.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="December" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,35 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A8BBA3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF4DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFA239"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +68,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,439 +444,469 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Time</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Meter 1</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Bypass</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Meter Blue</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Meter Red</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Steam Flow Meter</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Aspen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>08/10/25</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="2" t="n">
         <v>76</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>11/17/25</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>119524</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>29836</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>9836</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="2" t="n">
         <v>79969750</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>70959</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>11/19/25</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
         <v>119570</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
         <v>29845</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="2" t="n">
         <v>9855</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="2" t="n">
         <v>79996126</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="2" t="n">
         <v>70974</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>11/22/25</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
         <v>120003</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>29928</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>9941</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="2" t="n">
         <v>80268474</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="2" t="n">
         <v>71145</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>11/23/25</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
         <v>120371</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>30007</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>10017</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="2" t="n">
         <v>80517594</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="2" t="n">
         <v>71316</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>11/23/25</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
         <v>120372</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>30010</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>10019</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="2" t="n">
         <v>80518594</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="2" t="n">
         <v>71318</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>11/23/25</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
         <v>120373</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="2" t="n">
         <v>30012</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="2" t="n">
         <v>10019</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="2" t="n">
         <v>80519594</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="2" t="n">
         <v>71319</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>11/27/25</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
         <v>120379</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="2" t="n">
         <v>1300</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="2" t="n">
         <v>30025</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="2" t="n">
         <v>10025</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="2" t="n">
         <v>80520100</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="2" t="n">
         <v>71327</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>11/29/25</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="2" t="n">
         <v>94</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>11/30/25</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="2" t="n">
         <v>71</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="2" t="n">
         <v>33</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>12/01/25</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="2" t="n">
         <v>78</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>12/02/25</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="2" t="n">
         <v>68</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="2" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>12/03/25</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>06:00</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="2" t="n">
         <v>73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>-32</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>-26</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>